<commit_message>
Debug: Bunch of bug fixes and additional preloading so now most things load instantly.
</commit_message>
<xml_diff>
--- a/Spreadsheets/Opponent_Tracker.xlsx
+++ b/Spreadsheets/Opponent_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Pokemon TCG Legacy\Spreadsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FDD5FE-BEB5-4517-971D-9C9269848DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8092C0C7-F719-4DC8-8CD0-0A313EF3C7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14715" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="opponents_table" sheetId="1" r:id="rId1"/>
@@ -2622,9 +2622,6 @@
     <t>Spectator Pete</t>
   </si>
   <si>
-    <t>Deck Eruption</t>
-  </si>
-  <si>
     <t>CELESTE HARBOUR
 VERDANT FOREST
 8</t>
@@ -2648,6 +2645,9 @@
     <t>VERDANT FOREST
 GYM PLAZA
 12</t>
+  </si>
+  <si>
+    <t>REPLACE ME</t>
   </si>
 </sst>
 </file>
@@ -4279,31 +4279,31 @@
       <c r="AG1" s="198"/>
       <c r="AH1" s="199"/>
       <c r="AI1" s="163" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="AJ1" s="164"/>
       <c r="AK1" s="165"/>
       <c r="AL1" s="166"/>
       <c r="AM1" s="127" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="AN1" s="128"/>
       <c r="AO1" s="129"/>
       <c r="AP1" s="130"/>
       <c r="AQ1" s="127" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="AR1" s="128"/>
       <c r="AS1" s="129"/>
       <c r="AT1" s="130"/>
       <c r="AU1" s="127" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="AV1" s="128"/>
       <c r="AW1" s="129"/>
       <c r="AX1" s="130"/>
       <c r="AY1" s="127" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="AZ1" s="128"/>
       <c r="BA1" s="129"/>
@@ -13718,7 +13718,7 @@
         <v>8</v>
       </c>
       <c r="E119" t="s">
-        <v>857</v>
+        <v>862</v>
       </c>
       <c r="AM119" s="51"/>
       <c r="AO119" s="30" t="s">

</xml_diff>